<commit_message>
Texas developer entity pass: resolve 62 of 63 missing developer names
Pulled individual TDHCA Real Estate Analysis underwriting report PDFs
per application number to identify developer legal entities, including
a deeper full-document pull for 6 cases where the page-1 summary alone
was insufficient. Only Pathways at Santa Rita Courts West remains
unresolved (no company name printed anywhere in its source report).
</commit_message>
<xml_diff>
--- a/LIHTC_Master_Database_2025.xlsx
+++ b/LIHTC_Master_Database_2025.xlsx
@@ -44082,7 +44082,7 @@
       </c>
       <c r="D552" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>LCJ Development, Inc.</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
@@ -44122,7 +44122,7 @@
       </c>
       <c r="L552" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25038), source: https://www.tdhca.state.tx.us/readocs/uwrep/25038.pdf.</t>
         </is>
       </c>
       <c r="M552" t="inlineStr">
@@ -44162,7 +44162,7 @@
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>PK Development Group, LLC</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
@@ -44202,7 +44202,7 @@
       </c>
       <c r="L553" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25114), source: https://www.tdhca.state.tx.us/readocs/uwrep/25114.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M553" t="inlineStr">
@@ -44242,7 +44242,7 @@
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>PK Development Group, LLC</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
@@ -44282,7 +44282,7 @@
       </c>
       <c r="L554" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25118), source: https://www.tdhca.state.tx.us/readocs/uwrep/25118.pdf.</t>
         </is>
       </c>
       <c r="M554" t="inlineStr">
@@ -44322,7 +44322,7 @@
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Housing Developers, LLC</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
@@ -44362,7 +44362,7 @@
       </c>
       <c r="L555" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25170), source: https://www.tdhca.state.tx.us/readocs/uwrep/25170.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M555" t="inlineStr">
@@ -44402,7 +44402,7 @@
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Pecan Tree Square, LLC</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
@@ -44442,7 +44442,7 @@
       </c>
       <c r="L556" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25035), source: https://www.tdhca.state.tx.us/readocs/uwrep/25035.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M556" t="inlineStr">
@@ -44482,7 +44482,7 @@
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Belmont Development</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
@@ -44522,7 +44522,7 @@
       </c>
       <c r="L557" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25185), source: https://www.tdhca.state.tx.us/readocs/uwrep/25185.pdf.</t>
         </is>
       </c>
       <c r="M557" t="inlineStr">
@@ -44562,7 +44562,7 @@
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>National Church Residences</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
@@ -44602,7 +44602,7 @@
       </c>
       <c r="L558" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25093), source: https://www.tdhca.state.tx.us/readocs/uwrep/25093.pdf.</t>
         </is>
       </c>
       <c r="M558" t="inlineStr">
@@ -44642,7 +44642,7 @@
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Housing Developers, LLC</t>
         </is>
       </c>
       <c r="E559" t="inlineStr">
@@ -44682,7 +44682,7 @@
       </c>
       <c r="L559" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25171), source: https://www.tdhca.state.tx.us/readocs/uwrep/25171.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M559" t="inlineStr">
@@ -44722,7 +44722,7 @@
       </c>
       <c r="D560" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Housing Developers, LLC</t>
         </is>
       </c>
       <c r="E560" t="inlineStr">
@@ -44762,7 +44762,7 @@
       </c>
       <c r="L560" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25172), source: https://www.tdhca.state.tx.us/readocs/uwrep/25172.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M560" t="inlineStr">
@@ -44802,7 +44802,7 @@
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>National Church Residences</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
@@ -44842,7 +44842,7 @@
       </c>
       <c r="L561" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25072), source: https://www.tdhca.state.tx.us/readocs/uwrep/25072.pdf.</t>
         </is>
       </c>
       <c r="M561" t="inlineStr">
@@ -44882,7 +44882,7 @@
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>National Development of America, Inc</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
@@ -44922,7 +44922,7 @@
       </c>
       <c r="L562" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25204), source: https://www.tdhca.state.tx.us/readocs/uwrep/25204.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M562" t="inlineStr">
@@ -44962,7 +44962,7 @@
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Itex Group</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
@@ -45002,7 +45002,7 @@
       </c>
       <c r="L563" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25123), source: https://www.tdhca.state.tx.us/readocs/uwrep/25123.pdf.</t>
         </is>
       </c>
       <c r="M563" t="inlineStr">
@@ -45042,7 +45042,7 @@
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Mission Housing Development Corporation (MHDC)</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
@@ -45082,7 +45082,7 @@
       </c>
       <c r="L564" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25077); only Owner entity printed: Brownstone Affordable Housing, Ltd.; Mission Housing Development Corporation. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25077.pdf. Still requires manual follow-up. Developer entity refined 2026-06-30 via full-document review of TDHCA underwriting report (app #25077) — entity confirmed in Developer Fee/Sources&amp;Uses table, distinct from page-1 Key Principals box. Source: https://www.tdhca.state.tx.us/readocs/uwrep/25077.pdf.</t>
         </is>
       </c>
       <c r="M564" t="inlineStr">
@@ -45122,7 +45122,7 @@
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>National Church Residences</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
@@ -45162,7 +45162,7 @@
       </c>
       <c r="L565" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25107), source: https://www.tdhca.state.tx.us/readocs/uwrep/25107.pdf.</t>
         </is>
       </c>
       <c r="M565" t="inlineStr">
@@ -45202,7 +45202,7 @@
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Avenue U Development, LLC (95%)</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
@@ -45242,7 +45242,7 @@
       </c>
       <c r="L566" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25145), source: https://www.tdhca.state.tx.us/readocs/uwrep/25145.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M566" t="inlineStr">
@@ -45282,7 +45282,7 @@
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Woda Cooper Community III, LLC</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
@@ -45322,7 +45322,7 @@
       </c>
       <c r="L567" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25046), source: https://www.tdhca.state.tx.us/readocs/uwrep/25046.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M567" t="inlineStr">
@@ -45362,7 +45362,7 @@
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Verdite Developments LLC</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
@@ -45402,7 +45402,7 @@
       </c>
       <c r="L568" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25088), source: https://www.tdhca.state.tx.us/readocs/uwrep/25088.pdf.</t>
         </is>
       </c>
       <c r="M568" t="inlineStr">
@@ -45442,7 +45442,7 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Overland Property Group</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
@@ -45482,7 +45482,7 @@
       </c>
       <c r="L569" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25163), source: https://www.tdhca.state.tx.us/readocs/uwrep/25163.pdf.</t>
         </is>
       </c>
       <c r="M569" t="inlineStr">
@@ -45522,7 +45522,7 @@
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Denton Affordable Housing Corporation</t>
         </is>
       </c>
       <c r="E570" t="inlineStr">
@@ -45562,7 +45562,7 @@
       </c>
       <c r="L570" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25160), source: https://www.tdhca.state.tx.us/readocs/uwrep/26500_25160.pdf.</t>
         </is>
       </c>
       <c r="M570" t="inlineStr">
@@ -45602,7 +45602,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Overland Property Group</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
@@ -45642,7 +45642,7 @@
       </c>
       <c r="L571" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25164), source: https://www.tdhca.state.tx.us/readocs/uwrep/25164.pdf.</t>
         </is>
       </c>
       <c r="M571" t="inlineStr">
@@ -45682,7 +45682,7 @@
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>O-SDA Industries, LLC</t>
         </is>
       </c>
       <c r="E572" t="inlineStr">
@@ -45722,7 +45722,7 @@
       </c>
       <c r="L572" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25162), source: https://www.tdhca.state.tx.us/readocs/uwrep/25162.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M572" t="inlineStr">
@@ -45762,7 +45762,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Sycamore Strategies (10% Owner, 70% Developer)</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
@@ -45802,7 +45802,7 @@
       </c>
       <c r="L573" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25239), source: https://www.tdhca.state.tx.us/readocs/uwrep/25239.pdf.</t>
         </is>
       </c>
       <c r="M573" t="inlineStr">
@@ -45842,7 +45842,7 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Express Development, Inc</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
@@ -45882,7 +45882,7 @@
       </c>
       <c r="L574" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25175), source: https://www.tdhca.state.tx.us/readocs/uwrep/25175.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M574" t="inlineStr">
@@ -45922,7 +45922,7 @@
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>East 43rd St LLC (Co-Developer 50% Fee); JCM Ventures, LLC (Co-Developer 50% Fee)</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
@@ -45962,7 +45962,7 @@
       </c>
       <c r="L575" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25067), source: https://www.tdhca.state.tx.us/readocs/uwrep/25067.pdf.</t>
         </is>
       </c>
       <c r="M575" t="inlineStr">
@@ -46002,7 +46002,7 @@
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Brompton Development</t>
         </is>
       </c>
       <c r="E576" t="inlineStr">
@@ -46042,7 +46042,7 @@
       </c>
       <c r="L576" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25004), source: https://www.tdhca.state.tx.us/readocs/uwrep/25004.pdf.</t>
         </is>
       </c>
       <c r="M576" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Palladium McKinney Ranch Development, LLC</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
@@ -46122,7 +46122,7 @@
       </c>
       <c r="L577" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25116); only Owner entity printed: Palladium International S.a.r.l.; Casa Linda Development Corporation; Palladium USA, Inc.. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25116.pdf. Still requires manual follow-up. Developer entity refined 2026-06-30 via full-document review of TDHCA underwriting report (app #25116) — entity confirmed in Developer Fee/Sources&amp;Uses table, distinct from page-1 Key Principals box. Source: https://www.tdhca.state.tx.us/readocs/uwrep/25116.pdf.</t>
         </is>
       </c>
       <c r="M577" t="inlineStr">
@@ -46162,7 +46162,7 @@
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>PHP Development LLC (90% of fee); Auxano Development, LLC (10% of fee)</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
@@ -46202,7 +46202,7 @@
       </c>
       <c r="L578" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25022), source: https://www.tdhca.state.tx.us/readocs/uwrep/25022.pdf.</t>
         </is>
       </c>
       <c r="M578" t="inlineStr">
@@ -46242,7 +46242,7 @@
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Overland Property Group</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
@@ -46282,7 +46282,7 @@
       </c>
       <c r="L579" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25167), source: https://www.tdhca.state.tx.us/readocs/uwrep/25167.pdf.</t>
         </is>
       </c>
       <c r="M579" t="inlineStr">
@@ -46322,7 +46322,7 @@
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>PHP Development</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
@@ -46362,7 +46362,7 @@
       </c>
       <c r="L580" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25025), source: https://www.tdhca.state.tx.us/readocs/uwrep/25025.pdf.</t>
         </is>
       </c>
       <c r="M580" t="inlineStr">
@@ -46402,7 +46402,7 @@
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Banner Development</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
@@ -46442,7 +46442,7 @@
       </c>
       <c r="L581" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25133), source: https://www.tdhca.state.tx.us/readocs/uwrep/25133.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M581" t="inlineStr">
@@ -46482,7 +46482,7 @@
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>DMA Community Ventures II, LLC</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
@@ -46522,7 +46522,7 @@
       </c>
       <c r="L582" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25064), source: https://www.tdhca.state.tx.us/readocs/uwrep/25064.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M582" t="inlineStr">
@@ -46562,7 +46562,7 @@
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Overland Property Group</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
@@ -46602,7 +46602,7 @@
       </c>
       <c r="L583" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25165), source: https://www.tdhca.state.tx.us/readocs/uwrep/25165.pdf.</t>
         </is>
       </c>
       <c r="M583" t="inlineStr">
@@ -46642,7 +46642,7 @@
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Inter-Faith Housing Corporation</t>
         </is>
       </c>
       <c r="E584" t="inlineStr">
@@ -46682,7 +46682,7 @@
       </c>
       <c r="L584" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25128), source: https://www.tdhca.state.tx.us/readocs/uwrep/25128.pdf.</t>
         </is>
       </c>
       <c r="M584" t="inlineStr">
@@ -46722,7 +46722,7 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Windstone Developers, LLC</t>
         </is>
       </c>
       <c r="E585" t="inlineStr">
@@ -46762,7 +46762,7 @@
       </c>
       <c r="L585" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25031); only Owner entity printed: Nantucket Housing, LLC; Richco Rinehart Investments, LLC. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25031.pdf. Still requires manual follow-up. Developer entity refined 2026-06-30 via full-document review of TDHCA underwriting report (app #25031) — entity confirmed in Developer Fee/Sources&amp;Uses table, distinct from page-1 Key Principals box. Source: https://www.tdhca.state.tx.us/readocs/uwrep/25031.pdf.</t>
         </is>
       </c>
       <c r="M585" t="inlineStr">
@@ -46802,7 +46802,7 @@
       </c>
       <c r="D586" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Housing Developers, LLC (95% of fee); Broadleaf Development, LLC (5% of fee)</t>
         </is>
       </c>
       <c r="E586" t="inlineStr">
@@ -46842,7 +46842,7 @@
       </c>
       <c r="L586" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25150), source: https://www.tdhca.state.tx.us/readocs/uwrep/25150.pdf.</t>
         </is>
       </c>
       <c r="M586" t="inlineStr">
@@ -46882,7 +46882,7 @@
       </c>
       <c r="D587" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Brinshore Development, LLC</t>
         </is>
       </c>
       <c r="E587" t="inlineStr">
@@ -46922,7 +46922,7 @@
       </c>
       <c r="L587" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25178), source: https://www.tdhca.state.tx.us/readocs/uwrep/25178.pdf.</t>
         </is>
       </c>
       <c r="M587" t="inlineStr">
@@ -46962,7 +46962,7 @@
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Impact Residential Development, L.L.C.</t>
         </is>
       </c>
       <c r="E588" t="inlineStr">
@@ -47002,7 +47002,7 @@
       </c>
       <c r="L588" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25074), source: https://www.tdhca.state.tx.us/readocs/uwrep/25074.pdf.</t>
         </is>
       </c>
       <c r="M588" t="inlineStr">
@@ -47042,7 +47042,7 @@
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>CSH Silverleaf Senior Living GP, LLC</t>
         </is>
       </c>
       <c r="E589" t="inlineStr">
@@ -47082,7 +47082,7 @@
       </c>
       <c r="L589" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25126), source: https://www.tdhca.state.tx.us/readocs/uwrep/25126.pdf.</t>
         </is>
       </c>
       <c r="M589" t="inlineStr">
@@ -47122,7 +47122,7 @@
       </c>
       <c r="D590" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Impact Residential Development, L.L.C.</t>
         </is>
       </c>
       <c r="E590" t="inlineStr">
@@ -47162,7 +47162,7 @@
       </c>
       <c r="L590" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25073), source: https://www.tdhca.state.tx.us/readocs/uwrep/25073.pdf.</t>
         </is>
       </c>
       <c r="M590" t="inlineStr">
@@ -47202,7 +47202,7 @@
       </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Elizabeth Property Group</t>
         </is>
       </c>
       <c r="E591" t="inlineStr">
@@ -47242,7 +47242,7 @@
       </c>
       <c r="L591" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25201), source: https://www.tdhca.state.tx.us/readocs/uwrep/25201.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M591" t="inlineStr">
@@ -47282,7 +47282,7 @@
       </c>
       <c r="D592" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>O-SDA Industries, LLC</t>
         </is>
       </c>
       <c r="E592" t="inlineStr">
@@ -47322,7 +47322,7 @@
       </c>
       <c r="L592" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25158), source: https://www.tdhca.state.tx.us/readocs/uwrep/25158.pdf.</t>
         </is>
       </c>
       <c r="M592" t="inlineStr">
@@ -47362,7 +47362,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Foundation Communities</t>
         </is>
       </c>
       <c r="E593" t="inlineStr">
@@ -47402,7 +47402,7 @@
       </c>
       <c r="L593" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25187), source: https://www.tdhca.state.tx.us/readocs/uwrep/26501_25187.pdf.</t>
         </is>
       </c>
       <c r="M593" t="inlineStr">
@@ -47482,7 +47482,7 @@
       </c>
       <c r="L594" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25001); only Owner entity printed: none. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25001.pdf. Still requires manual follow-up. Re-checked 2026-06-30 via full 15-page document review (not just page 1) — confirmed no developer legal entity is stated anywhere in the report; Developer role is assigned to a named individual (Suzanne Schwertner) with no company affiliation printed. Requires direct TDHCA/HACA contact.</t>
         </is>
       </c>
       <c r="M594" t="inlineStr">
@@ -47522,7 +47522,7 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Linville Capital</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
@@ -47562,7 +47562,7 @@
       </c>
       <c r="L595" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25066), source: https://www.tdhca.state.tx.us/readocs/uwrep/25066.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M595" t="inlineStr">
@@ -47602,7 +47602,7 @@
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Madhouse Development, Inc</t>
         </is>
       </c>
       <c r="E596" t="inlineStr">
@@ -47642,7 +47642,7 @@
       </c>
       <c r="L596" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25217), source: https://www.tdhca.state.tx.us/readocs/uwrep/25217.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M596" t="inlineStr">
@@ -47682,7 +47682,7 @@
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Rea Ventures Group LLC</t>
         </is>
       </c>
       <c r="E597" t="inlineStr">
@@ -47722,7 +47722,7 @@
       </c>
       <c r="L597" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25060); only Owner entity printed: Rea GP Holdings Group IV, LLC; Austin Stone, LLC. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25060.pdf. Still requires manual follow-up. Developer entity refined 2026-06-30 via full-document review of TDHCA underwriting report (app #25060) — entity confirmed in Developer Fee/Sources&amp;Uses table, distinct from page-1 Key Principals box. Source: https://www.tdhca.state.tx.us/readocs/uwrep/25060.pdf.</t>
         </is>
       </c>
       <c r="M597" t="inlineStr">
@@ -47762,7 +47762,7 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>GHT Development II, LLC and Urbanize Inc.</t>
         </is>
       </c>
       <c r="E598" t="inlineStr">
@@ -47802,7 +47802,7 @@
       </c>
       <c r="L598" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity not stated on underwriting report page 1 (app #25112); only Owner entity printed: Generation Housing Development, LLC; White Rock Residential, LLC; Hill Tide Ventures, LLC. Re-checked 2026-06-30 via TDHCA Real Estate Analysis report, source: https://www.tdhca.state.tx.us/readocs/uwrep/25112.pdf. Still requires manual follow-up. Developer entity refined 2026-06-30 via full-document review of TDHCA underwriting report (app #25112) — entity confirmed in Developer Fee/Sources&amp;Uses table, distinct from page-1 Key Principals box. Source: https://www.tdhca.state.tx.us/readocs/uwrep/25112.pdf.</t>
         </is>
       </c>
       <c r="M598" t="inlineStr">
@@ -47842,7 +47842,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>NRP Lone Star Development LLC (80% of fee); Community Housing Resource Partners, Inc. (20% of fee)</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
@@ -47882,7 +47882,7 @@
       </c>
       <c r="L599" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25070), source: https://www.tdhca.state.tx.us/readocs/uwrep/25070.pdf.</t>
         </is>
       </c>
       <c r="M599" t="inlineStr">
@@ -47922,7 +47922,7 @@
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>G2 Equity Inc.</t>
         </is>
       </c>
       <c r="E600" t="inlineStr">
@@ -47962,7 +47962,7 @@
       </c>
       <c r="L600" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25177), source: https://www.tdhca.state.tx.us/readocs/uwrep/25177.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M600" t="inlineStr">
@@ -48002,7 +48002,7 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Danco Communities</t>
         </is>
       </c>
       <c r="E601" t="inlineStr">
@@ -48042,7 +48042,7 @@
       </c>
       <c r="L601" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25013), source: https://www.tdhca.state.tx.us/readocs/uwrep/25013.pdf.</t>
         </is>
       </c>
       <c r="M601" t="inlineStr">
@@ -48082,7 +48082,7 @@
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Roundstone Development, LLC</t>
         </is>
       </c>
       <c r="E602" t="inlineStr">
@@ -48122,7 +48122,7 @@
       </c>
       <c r="L602" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25055), source: https://www.tdhca.state.tx.us/readocs/uwrep/25055.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M602" t="inlineStr">
@@ -48162,7 +48162,7 @@
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Roundstone Development, LLC</t>
         </is>
       </c>
       <c r="E603" t="inlineStr">
@@ -48202,7 +48202,7 @@
       </c>
       <c r="L603" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25051), source: https://www.tdhca.state.tx.us/readocs/uwrep/25051.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M603" t="inlineStr">
@@ -48242,7 +48242,7 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Madhouse Development, Inc. (75% of fee)</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
@@ -48282,7 +48282,7 @@
       </c>
       <c r="L604" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25214), source: https://www.tdhca.state.tx.us/readocs/uwrep/25214.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M604" t="inlineStr">
@@ -48322,7 +48322,7 @@
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Versa Development, LLC (Co-Developer 50% Fee); Brownsville Housing Opportunity Corporation (Co-Developer 50% Fee)</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
@@ -48362,7 +48362,7 @@
       </c>
       <c r="L605" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25196), source: https://www.tdhca.state.tx.us/readocs/uwrep/25196.pdf.</t>
         </is>
       </c>
       <c r="M605" t="inlineStr">
@@ -48402,7 +48402,7 @@
       </c>
       <c r="D606" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>G2 Equity Inc. (90%)</t>
         </is>
       </c>
       <c r="E606" t="inlineStr">
@@ -48442,7 +48442,7 @@
       </c>
       <c r="L606" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25271), source: https://www.tdhca.state.tx.us/readocs/uwrep/25271.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M606" t="inlineStr">
@@ -48482,7 +48482,7 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Paisano Housing Redevelopment Corporation (PHRC)</t>
         </is>
       </c>
       <c r="E607" t="inlineStr">
@@ -48522,7 +48522,7 @@
       </c>
       <c r="L607" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25270), source: https://www.tdhca.state.tx.us/readocs/uwrep/25270.pdf.</t>
         </is>
       </c>
       <c r="M607" t="inlineStr">
@@ -77627,7 +77627,7 @@
       </c>
       <c r="D976" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>PHP Development LLC (90% of fee); Auxano Development, LLC (10% of fee)</t>
         </is>
       </c>
       <c r="E976" t="inlineStr">
@@ -77657,7 +77657,7 @@
       </c>
       <c r="L976" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25017), source: https://www.tdhca.state.tx.us/readocs/uwrep/25017.pdf.</t>
         </is>
       </c>
       <c r="M976" t="inlineStr">
@@ -77697,7 +77697,7 @@
       </c>
       <c r="D977" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Sycamore Strategies</t>
         </is>
       </c>
       <c r="E977" t="inlineStr">
@@ -77727,7 +77727,7 @@
       </c>
       <c r="L977" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25240), source: https://www.tdhca.state.tx.us/readocs/uwrep/25240.pdf. NOTE: role label (Owner vs Developer) not explicitly printed on source page 1; entity assignment inferred from naming convention/context - recommend verification against full report if used for official purposes.</t>
         </is>
       </c>
       <c r="M977" t="inlineStr">
@@ -77767,7 +77767,7 @@
       </c>
       <c r="D978" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Trinity Housing Development</t>
         </is>
       </c>
       <c r="E978" t="inlineStr">
@@ -77797,7 +77797,7 @@
       </c>
       <c r="L978" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25261), source: https://www.tdhca.state.tx.us/readocs/uwrep/25261.pdf.</t>
         </is>
       </c>
       <c r="M978" t="inlineStr">
@@ -77837,7 +77837,7 @@
       </c>
       <c r="D979" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>The NHP Foundation (SLP, 72% Developer); Trinity East Village CDC (SLP, 18% Developer); Victory Redevelopment (100% GP, 10% Developer)</t>
         </is>
       </c>
       <c r="E979" t="inlineStr">
@@ -77867,7 +77867,7 @@
       </c>
       <c r="L979" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25090), source: https://www.tdhca.state.tx.us/readocs/uwrep/25090.pdf.</t>
         </is>
       </c>
       <c r="M979" t="inlineStr">
@@ -77907,7 +77907,7 @@
       </c>
       <c r="D980" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Texas Housing Developers, LLC (100% of fee)</t>
         </is>
       </c>
       <c r="E980" t="inlineStr">
@@ -77937,7 +77937,7 @@
       </c>
       <c r="L980" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25155), source: https://www.tdhca.state.tx.us/readocs/uwrep/25155.pdf.</t>
         </is>
       </c>
       <c r="M980" t="inlineStr">
@@ -77977,7 +77977,7 @@
       </c>
       <c r="D981" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>NRP Lone Star Development LLC (80% of fee); Community Housing Resource Partners, Inc. (20% of fee)</t>
         </is>
       </c>
       <c r="E981" t="inlineStr">
@@ -78007,7 +78007,7 @@
       </c>
       <c r="L981" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25071), source: https://www.tdhca.state.tx.us/readocs/uwrep/25071.pdf.</t>
         </is>
       </c>
       <c r="M981" t="inlineStr">
@@ -78047,7 +78047,7 @@
       </c>
       <c r="D982" t="inlineStr">
         <is>
-          <t>Not Available - contact name only in source</t>
+          <t>Green Mills Group</t>
         </is>
       </c>
       <c r="E982" t="inlineStr">
@@ -78077,7 +78077,7 @@
       </c>
       <c r="L982" t="inlineStr">
         <is>
-          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project).</t>
+          <t>FINAL award per TDHCA 2025 9% HTC Award and Waiting List Recommendations, version date October 14, 2025 (confirmed by TDHCA Governing Board action; held per 10 TAC Section 11.6(4) until September 30, 2025). Source only lists contact names, not developer entity names - developer field requires follow-up (would need individual TDHCA underwriting reports per project). Developer entity name added 2026-06-30 from TDHCA Real Estate Analysis underwriting report (app #25016), source: https://www.tdhca.state.tx.us/readocs/uwrep/25016.pdf.</t>
         </is>
       </c>
       <c r="M982" t="inlineStr">

</xml_diff>